<commit_message>
Answer workbooks: taller note rows so explanations are not clipped
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/practice/answers/q011.xlsx
+++ b/practice/answers/q011.xlsx
@@ -1972,14 +1972,14 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
+    <row r="6" ht="64" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>(b) The mean (33.9) sits below the median (35.5). When the mean is pulled below the median, the distribution has a longer left tail: a group of RMs with unusually low canola yields drags the mean down while barely moving the median.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1">
+    <row r="7" ht="64" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>(c) The median. Half the RMs sit above 35.5 and half below, and it ignores the badly hit low tail; the mean is dragged 1.6 bushels below that by the worst RMs, so it understates a typical RM.</t>

</xml_diff>

<commit_message>
Apply the 12 agent reviews: workbook fixes, bank wording; module 2 compliance pass
Two Fable and two Opus reviewers per five questions verified every
Q1-30 answer workbook against independent recomputation. Fixes: Q3
copies values instead of linking, Q5 one-decimal fractions, Q6 note
names the cell to reformat, Q9 grand total moved out of the header
row, Q10 counts explained per function, Q11 parts reordered so the
judgment follows the statistics, Q12 matching ranges, Q15/Q19/Q20
note precision, Q17 per-year data sheets, legend colours now match
cells everywhere, drought language tempered. Module 2 bank: fictional
classmates recast second-person, Q35 mangled sentence and typos fixed.
Review reports in reviews/module01_answer_check/.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/practice/answers/q011.xlsx
+++ b/practice/answers/q011.xlsx
@@ -44,7 +44,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
+        <fgColor rgb="00CFE2F3"/>
       </patternFill>
     </fill>
     <fill>
@@ -54,7 +54,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFE2F3"/>
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,8 +83,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1953,7 +1953,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Standard deviation (d)</t>
+          <t>Standard deviation (c)</t>
         </is>
       </c>
       <c r="B3" s="3">
@@ -1964,7 +1964,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>IQR (d)</t>
+          <t>IQR (c)</t>
         </is>
       </c>
       <c r="B4" s="3">
@@ -1982,7 +1982,7 @@
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>(c) The median. Half the RMs sit above 35.5 and half below, and it ignores the badly hit low tail; the mean is dragged 1.6 bushels below that by the worst RMs, so it understates a typical RM.</t>
+          <t>(d) The median. Half the RMs sit above 35.5 and half below, and it ignores the badly hit low tail; the mean is dragged 1.6 bushels below that by the worst RMs, so it understates a typical RM.</t>
         </is>
       </c>
     </row>

</xml_diff>